<commit_message>
update database with c3mechlite
</commit_message>
<xml_diff>
--- a/data/database/2026-09-14-database-mechanisms-H2-NH3-preliminary.xlsx
+++ b/data/database/2026-09-14-database-mechanisms-H2-NH3-preliminary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\PhD-ULB\Programming\2026-AI-agent-combustion\data\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FC98855-5FFE-4F1C-95AE-F74F225729B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32BCF310-F95B-4DFC-8B5B-F45B8CDB8B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{A09D45FC-1E38-41D2-9517-F3EDE489635B}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="202">
   <si>
     <t>ID</t>
   </si>
@@ -654,6 +654,12 @@
   </si>
   <si>
     <t>lean, stability</t>
+  </si>
+  <si>
+    <t>autoignition, ignition, IDT</t>
+  </si>
+  <si>
+    <t>C3MechLiteV4.0.1</t>
   </si>
 </sst>
 </file>
@@ -3255,7 +3261,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A6FBBD4-7673-49DB-9D2F-7AC74B944568}">
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="32.6328125" customWidth="1"/>
@@ -4207,6 +4213,47 @@
         <v>193</v>
       </c>
     </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A24" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="E24" s="2">
+        <v>1100</v>
+      </c>
+      <c r="F24" s="2">
+        <v>1500</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="I24" s="2">
+        <v>1</v>
+      </c>
+      <c r="J24" s="2">
+        <v>30</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>